<commit_message>
fix(timesheet): drop June's autofilter and filter names, size the X row as a code row
</commit_message>
<xml_diff>
--- a/backend/templates/GSSG-HR_Monthly_Time_Sheet.xlsx
+++ b/backend/templates/GSSG-HR_Monthly_Time_Sheet.xlsx
@@ -9,13 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_parts" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="Z_1A0407EF_5AB1_4F3F_8A5E_B19751176730_.wvu.FilterData" localSheetId="0" hidden="1">Sheet1!$D$5:$E$290</definedName>
-    <definedName name="Z_98E4907F_34A1_48C9_9DCA_73702E5AE537_.wvu.FilterData" localSheetId="0" hidden="1">Sheet1!$A$5:$E$290</definedName>
-    <definedName name="Z_CD164567_4829_46B0_AEED_42A99E823C5A_.wvu.FilterData" localSheetId="0" hidden="1">Sheet1!$D$5:$E$290</definedName>
-    <definedName name="Z_DBA20609_2CD4_449D_B1CD_3710B41950FA_.wvu.FilterData" localSheetId="0" hidden="1">Sheet1!$D$5:$E$290</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$D$5:$E$290</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2146,7 +2140,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D5:E290"/>
   <mergeCells count="15">
     <mergeCell ref="D3:P3"/>
     <mergeCell ref="AJ2:AK2"/>
@@ -2530,7 +2523,7 @@
       </c>
       <c r="E19" s="12" t="n"/>
     </row>
-    <row r="20" ht="39.95" customHeight="1" s="84">
+    <row r="20" ht="35.1" customHeight="1" s="84">
       <c r="A20" s="78" t="n"/>
       <c r="B20" s="70" t="n"/>
       <c r="C20" s="11" t="inlineStr">

</xml_diff>

<commit_message>
fix(timesheet): add subsequent-row specimen so the header rule draws once
</commit_message>
<xml_diff>
--- a/backend/templates/GSSG-HR_Monthly_Time_Sheet.xlsx
+++ b/backend/templates/GSSG-HR_Monthly_Time_Sheet.xlsx
@@ -2216,6 +2216,50 @@
       <c r="AO1" s="31" t="n"/>
       <c r="AP1" s="29" t="n"/>
     </row>
+    <row r="2" ht="27.95" customHeight="1" s="84">
+      <c r="A2" s="41" t="n"/>
+      <c r="B2" s="34" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="36" t="n"/>
+      <c r="E2" s="36" t="n"/>
+      <c r="F2" s="50" t="n"/>
+      <c r="G2" s="50" t="n"/>
+      <c r="H2" s="50" t="n"/>
+      <c r="I2" s="50" t="n"/>
+      <c r="J2" s="50" t="n"/>
+      <c r="K2" s="50" t="n"/>
+      <c r="L2" s="50" t="n"/>
+      <c r="M2" s="50" t="n"/>
+      <c r="N2" s="50" t="n"/>
+      <c r="O2" s="50" t="n"/>
+      <c r="P2" s="50" t="n"/>
+      <c r="Q2" s="50" t="n"/>
+      <c r="R2" s="50" t="n"/>
+      <c r="S2" s="50" t="n"/>
+      <c r="T2" s="50" t="n"/>
+      <c r="U2" s="50" t="n"/>
+      <c r="V2" s="50" t="n"/>
+      <c r="W2" s="50" t="n"/>
+      <c r="X2" s="50" t="n"/>
+      <c r="Y2" s="50" t="n"/>
+      <c r="Z2" s="50" t="n"/>
+      <c r="AA2" s="50" t="n"/>
+      <c r="AB2" s="20" t="n"/>
+      <c r="AC2" s="20" t="n"/>
+      <c r="AD2" s="20" t="n"/>
+      <c r="AE2" s="20" t="n"/>
+      <c r="AF2" s="20" t="n"/>
+      <c r="AG2" s="20" t="n"/>
+      <c r="AH2" s="20" t="n"/>
+      <c r="AI2" s="20" t="n"/>
+      <c r="AJ2" s="52" t="n"/>
+      <c r="AK2" s="26" t="n"/>
+      <c r="AL2" s="17" t="n"/>
+      <c r="AM2" s="17" t="n"/>
+      <c r="AN2" s="28" t="n"/>
+      <c r="AO2" s="32" t="n"/>
+      <c r="AP2" s="30" t="n"/>
+    </row>
     <row r="3" ht="27.95" customHeight="1" s="84">
       <c r="A3" s="79" t="inlineStr">
         <is>

</xml_diff>